<commit_message>
botones de subir a server
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO.xlsx
+++ b/SEGUIMIENTO.xlsx
@@ -148,7 +148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -170,11 +170,55 @@
         <color rgb="00B8C4D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B8C4D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B8C4D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B8C4D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B8C4D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B8C4D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B8C4D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B8C4D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B8C4D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -308,6 +352,9 @@
     <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -673,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -752,11 +799,11 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>46249</v>
+        <v>46257</v>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>22 días desde el pago</t>
+          <t>30 dias desde el pago</t>
         </is>
       </c>
     </row>
@@ -766,7 +813,9 @@
           <t>Tarifa por hora (rellenar)</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
+      <c r="C9" s="7" t="n">
+        <v>20</v>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>← escribe aquí tu tarifa; los importes se calculan solos</t>
@@ -820,14 +869,14 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>BC-1, BC-2</t>
+          <t>BC-1, BC-2, BC-3, ADM</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>3830</v>
+        <v>3920</v>
       </c>
       <c r="F13" s="12">
         <f>SUMIFS(Sesiones!$D:$D,Sesiones!$B:$B,"BC",Sesiones!$A:$A,"&gt;="&amp;DATE(2026,7,24))</f>
@@ -870,10 +919,8 @@
           <t>TOTAL PROYECTO</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C15" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="D15" s="20">
         <f>SUM(D13:D14)</f>
@@ -895,7 +942,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>⚠  Las horas están a 0 porque nunca se registraron: este control se creó el 2026-08-15. Las líneas de código y los días de actividad sí son datos reales sacados de git.</t>
+          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una) a partir de las marcas de tiempo de los archivos y del volumen de los commits: son estimaciones documentadas, no cronometro. Las del 15 y 16 de agosto estan registradas. Total pendiente de facturar: 19,0 h = 380 EUR.</t>
         </is>
       </c>
     </row>
@@ -986,6 +1033,11 @@
           <t>El bloque BC-2 está escrito sobre 'develop', que no incluye BC-1. El commit d4a4709 borró CameraController.kt, archivo que BC-2 modifica. Integrarlo en 'main' no será un merge limpio.</t>
         </is>
       </c>
+      <c r="D26" s="55" t="n"/>
+      <c r="E26" s="55" t="n"/>
+      <c r="F26" s="55" t="n"/>
+      <c r="G26" s="55" t="n"/>
+      <c r="H26" s="56" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="25" t="inlineStr">
@@ -998,6 +1050,11 @@
           <t>BC-2 (~2803 líneas, el bloque más grande) sigue sin commitear.</t>
         </is>
       </c>
+      <c r="D27" s="55" t="n"/>
+      <c r="E27" s="55" t="n"/>
+      <c r="F27" s="55" t="n"/>
+      <c r="G27" s="55" t="n"/>
+      <c r="H27" s="56" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="25" t="inlineStr">
@@ -1008,6 +1065,69 @@
       <c r="C28" s="26" t="inlineStr">
         <is>
           <t>BC-2 es medición previa al cifrado, no una funcionalidad terminada. Convendría facturarlo como investigación, no como feature entregada.</t>
+        </is>
+      </c>
+      <c r="D28" s="55" t="n"/>
+      <c r="E28" s="55" t="n"/>
+      <c r="F28" s="55" t="n"/>
+      <c r="G28" s="55" t="n"/>
+      <c r="H28" s="56" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>OBJETIVO DE FACTURACION — cierre de septiembre 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Registrado a 2026-08-23</t>
+        </is>
+      </c>
+      <c r="C31">
+        <f>Resumen!C23</f>
+        <v/>
+      </c>
+      <c r="D31">
+        <f>C31*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Objetivo minimo (horas / importe)</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>100</v>
+      </c>
+      <c r="D32">
+        <f>C32*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pendiente de generar</t>
+        </is>
+      </c>
+      <c r="C33">
+        <f>C32-C31</f>
+        <v/>
+      </c>
+      <c r="D33">
+        <f>C33*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>A 30 h/semana las horas restantes se cubren en ~2,7 semanas: el umbral de 2000 EUR se cruza alrededor del jueves 10 de septiembre de 2026. La ventana 24-ago -&gt; 30-sep (5 semanas + 3 dias) da capacidad para 168 h = hasta 187 h acumuladas = 3740 EUR.</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1232,9 @@
           <t>BC-1</t>
         </is>
       </c>
-      <c r="D4" s="27" t="n"/>
+      <c r="D4" s="27" t="n">
+        <v>6</v>
+      </c>
       <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Grabación continua: EvidenceStore (buffer en anillo, pre-roll 120 s, segmentos 8 MB), reescritura de RecordingActivity, retirada de CameraController</t>
@@ -1148,10 +1270,12 @@
           <t>BC-2</t>
         </is>
       </c>
-      <c r="D5" s="27" t="n"/>
+      <c r="D5" s="27" t="n">
+        <v>6</v>
+      </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>Cifrado (medición): CryptoBenchmark (SHA-256 + AES-256-GCM por bloques), RecorderWatch (watchdog de grabaciones largas), endpoint /benchmark, fix de path traversal, 2 scripts Python</t>
+          <t>Cifrado (medicion): CryptoBenchmark (SHA-256 + AES-256-GCM por bloques), RecorderWatch (watchdog de grabaciones largas), endpoint /benchmark, fix de path traversal, 2 scripts Python, testing con videos reales</t>
         </is>
       </c>
       <c r="F5" s="29" t="inlineStr">
@@ -1180,7 +1304,9 @@
         </is>
       </c>
       <c r="C6" s="10" t="n"/>
-      <c r="D6" s="27" t="n"/>
+      <c r="D6" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
           <t>Alta del sistema de seguimiento de horas (cubre las dos apps)</t>
@@ -1202,45 +1328,149 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="28" t="n"/>
-      <c r="F7" s="31" t="n"/>
-      <c r="G7" s="31" t="n"/>
-      <c r="H7" s="31" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="32" t="n"/>
-      <c r="B8" s="15" t="n"/>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="33" t="n"/>
-      <c r="F8" s="34" t="n"/>
-      <c r="G8" s="34" t="n"/>
-      <c r="H8" s="34" t="n"/>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>BC-3</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>Pantalla en reposo al grabar + cronometro en RecordingActivity. Compilado y desplegado en la unidad</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>Horas imputadas en la sesion del 2026-08-16 (bloque BC-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="32" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>BC-2</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>Cifrado (medicion): CryptoBenchmark (SHA-256 + AES-256-GCM por bloques) CONTINUACION</t>
+        </is>
+      </c>
+      <c r="F8" s="50" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="57" t="inlineStr">
+        <is>
+          <t>Registrado</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="31" t="n"/>
-      <c r="G9" s="31" t="n"/>
-      <c r="H9" s="31" t="n"/>
+      <c r="A9" s="32" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>BC-1</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>Funcionalidad Subir a servidor yes/no, visualizacion de tiempo de grabacion</t>
+        </is>
+      </c>
+      <c r="F9" s="50" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="57" t="inlineStr">
+        <is>
+          <t>Registrado</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="n"/>
-      <c r="B10" s="15" t="n"/>
+      <c r="A10" s="32" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
       <c r="C10" s="15" t="n"/>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="34" t="n"/>
-      <c r="G10" s="34" t="n"/>
-      <c r="H10" s="34" t="n"/>
+      <c r="D10" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>Reuniones semana del 17 agosto al 21</t>
+        </is>
+      </c>
+      <c r="F10" s="50" t="n"/>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="57" t="inlineStr">
+        <is>
+          <t>Registrado</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -1618,7 +1848,7 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="B4:B46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Aplicación" prompt="BC = BodyCamServer  ·  AN = AeriaNexusPrototype" type="list">
       <formula1>"BC,AN"</formula1>
     </dataValidation>
@@ -1627,6 +1857,9 @@
     </dataValidation>
     <dataValidation sqref="G4:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BC-1,BC-2,BC-3,BC-4,AN-1,AN-2,ADM"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1639,7 +1872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1798,108 +2031,192 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="n"/>
-      <c r="B6" s="39" t="n"/>
-      <c r="C6" s="40" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>BC-3</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>Pantalla en reposo + cronometro</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>Sin commitear (develop)</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="12">
+        <f>SUMIF(Sesiones!$C:$C,A6,Sesiones!$D:$D)</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>I6*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>ADM</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Administracion (seguimiento de horas)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>Continuo</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="12">
+        <f>SUMIF(Sesiones!$C:$C,A7,Sesiones!$D:$D)</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>I7*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="39" t="n"/>
+      <c r="B8" s="39" t="n"/>
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>Subtotal BodyCamServer</t>
         </is>
       </c>
-      <c r="D6" s="39" t="n"/>
-      <c r="E6" s="39" t="n"/>
-      <c r="F6" s="41">
-        <f>SUM(F4:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="42">
-        <f>SUM(G4:G5)</f>
-        <v/>
-      </c>
-      <c r="H6" s="42">
-        <f>SUM(H4:H5)</f>
-        <v/>
-      </c>
-      <c r="I6" s="43">
-        <f>SUM(I4:I5)</f>
-        <v/>
-      </c>
-      <c r="J6" s="44">
-        <f>SUM(J4:J5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="D8" s="39" t="n"/>
+      <c r="E8" s="39" t="n"/>
+      <c r="F8" s="41">
+        <f>SUM(F4:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="42">
+        <f>SUM(G4:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="42">
+        <f>SUM(H4:H7)</f>
+        <v/>
+      </c>
+      <c r="I8" s="43">
+        <f>SUM(I4:I7)</f>
+        <v/>
+      </c>
+      <c r="J8" s="44">
+        <f>SUM(J4:J7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>AN</t>
         </is>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>AeriaNexusPrototype</t>
         </is>
       </c>
-      <c r="C8" s="45" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>Sin bloques posteriores al pago</t>
         </is>
       </c>
-      <c r="D8" s="31" t="n"/>
-      <c r="E8" s="37" t="inlineStr">
+      <c r="D10" s="31" t="n"/>
+      <c r="E10" s="37" t="inlineStr">
         <is>
           <t>Al día</t>
         </is>
       </c>
-      <c r="F8" s="46" t="n">
+      <c r="F10" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I10" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="13">
-        <f>I8*Resumen!$C$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="47" t="n"/>
-      <c r="B10" s="47" t="n"/>
-      <c r="C10" s="48" t="inlineStr">
+      <c r="J10" s="13">
+        <f>I10*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="n"/>
+      <c r="B12" s="47" t="n"/>
+      <c r="C12" s="48" t="inlineStr">
         <is>
           <t>TOTAL PROYECTO</t>
         </is>
       </c>
-      <c r="D10" s="47" t="n"/>
-      <c r="E10" s="47" t="n"/>
-      <c r="F10" s="49">
-        <f>SUM(F4:F5)+F8</f>
-        <v/>
-      </c>
-      <c r="G10" s="21">
-        <f>SUM(G4:G5)+G8</f>
-        <v/>
-      </c>
-      <c r="H10" s="21">
-        <f>SUM(H4:H5)+H8</f>
-        <v/>
-      </c>
-      <c r="I10" s="22">
-        <f>SUM(I4:I5)+I8</f>
-        <v/>
-      </c>
-      <c r="J10" s="23">
-        <f>SUM(J4:J5)+J8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="D12" s="47" t="n"/>
+      <c r="E12" s="47" t="n"/>
+      <c r="F12" s="49">
+        <f>SUM(F4:F7)+F10</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>SUM(G4:G7)+G10</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>SUM(H4:H7)+H10</f>
+        <v/>
+      </c>
+      <c r="I12" s="22">
+        <f>SUM(I4:I7)+I10</f>
+        <v/>
+      </c>
+      <c r="J12" s="23">
+        <f>SUM(J4:J7)+J10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Las columnas 'Horas' e 'Importe' se calculan solas a partir de la hoja Sesiones. No escribas en ellas.</t>
         </is>
@@ -1908,7 +2225,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A14:J14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
pre buffer integrado, let azul y armar al abrir la app
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO.xlsx
+++ b/SEGUIMIENTO.xlsx
@@ -869,14 +869,14 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>BC-1, BC-2, BC-3, ADM</t>
+          <t>BC-1, BC-2, BC-3, BC-4, ADM</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>3920</v>
+        <v>4900</v>
       </c>
       <c r="F13" s="12">
         <f>SUMIFS(Sesiones!$D:$D,Sesiones!$B:$B,"BC",Sesiones!$A:$A,"&gt;="&amp;DATE(2026,7,24))</f>
@@ -942,7 +942,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una) a partir de las marcas de tiempo de los archivos y del volumen de los commits: son estimaciones documentadas, no cronometro. Las del 15 y 16 de agosto estan registradas. Total pendiente de facturar: 19,0 h = 380 EUR.</t>
+          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una) a partir de las marcas de tiempo de los archivos y del volumen de los commits. Del 15 de agosto en adelante estan registradas en tiempo real. Total pendiente de facturar: 21,2 h = 424 EUR.</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1042,12 @@
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>⚠ SIN ENTREGAR</t>
+          <t>OK - ARBOL LIMPIO</t>
         </is>
       </c>
       <c r="C27" s="26" t="inlineStr">
         <is>
-          <t>BC-2 (~2803 líneas, el bloque más grande) sigue sin commitear.</t>
+          <t>Todo commiteado en develop a 2026-08-23: db04e55 y a599da9. Lo que queda pendiente es integrar develop y main, que han divergido.</t>
         </is>
       </c>
       <c r="D27" s="55" t="n"/>
@@ -1473,24 +1473,76 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="28" t="n"/>
-      <c r="F11" s="31" t="n"/>
-      <c r="G11" s="31" t="n"/>
-      <c r="H11" s="31" t="n"/>
+      <c r="A11" s="32" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>Analisis del Security Feature List (34 features: 15 viables sin backend, 12 parciales, 7 bloqueadas), ruta de desarrollo hasta fin de septiembre y actualizacion del seguimiento</t>
+        </is>
+      </c>
+      <c r="F11" s="50" t="inlineStr">
+        <is>
+          <t>db04e55</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="57" t="inlineStr">
+        <is>
+          <t>Marcas de tiempo 15:52-16:16</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="n"/>
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="34" t="n"/>
-      <c r="G12" s="34" t="n"/>
-      <c r="H12" s="34" t="n"/>
+      <c r="A12" s="32" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>BC-4</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>Panel de control: 3 bugs de la pregunta de envio (finish() en paradas redundantes, rebote de F2, arranque de grabacion con la pregunta abierta), rediseno para pantalla de 3 cm con iconos vectoriales, migracion de las dos pantallas a Compose con 8 previews, fullscreen real (tema, inmersivo, insets del decor)</t>
+        </is>
+      </c>
+      <c r="F12" s="50" t="inlineStr">
+        <is>
+          <t>db04e55, a599da9</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="57" t="inlineStr">
+        <is>
+          <t>Marcas de tiempo 16:16-18:04</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -1872,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2115,108 +2167,153 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="39" t="n"/>
-      <c r="B8" s="39" t="n"/>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>BC-4</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>Panel de control (UX + Compose)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46257</v>
+      </c>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>En develop (db04e55, a599da9)</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="n">
+        <v>16</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>978</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>329</v>
+      </c>
+      <c r="I8" s="12">
+        <f>SUMIF(Sesiones!$C:$C,A8,Sesiones!$D:$D)</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>I8*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="39" t="n"/>
+      <c r="B9" s="39" t="n"/>
+      <c r="C9" s="40" t="inlineStr">
         <is>
           <t>Subtotal BodyCamServer</t>
         </is>
       </c>
-      <c r="D8" s="39" t="n"/>
-      <c r="E8" s="39" t="n"/>
-      <c r="F8" s="41">
-        <f>SUM(F4:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="42">
-        <f>SUM(G4:G7)</f>
-        <v/>
-      </c>
-      <c r="H8" s="42">
-        <f>SUM(H4:H7)</f>
-        <v/>
-      </c>
-      <c r="I8" s="43">
-        <f>SUM(I4:I7)</f>
-        <v/>
-      </c>
-      <c r="J8" s="44">
-        <f>SUM(J4:J7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="41">
+        <f>SUM(F4:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="42">
+        <f>SUM(G4:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="42">
+        <f>SUM(H4:H8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="43">
+        <f>SUM(I4:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="44">
+        <f>SUM(J4:J8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>AN</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>AeriaNexusPrototype</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>Sin bloques posteriores al pago</t>
         </is>
       </c>
-      <c r="D10" s="31" t="n"/>
-      <c r="E10" s="37" t="inlineStr">
+      <c r="D11" s="31" t="n"/>
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>Al día</t>
         </is>
       </c>
-      <c r="F10" s="46" t="n">
+      <c r="F11" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I11" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J11" s="13">
         <f>I10*Resumen!$C$9</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="47" t="n"/>
-      <c r="B12" s="47" t="n"/>
-      <c r="C12" s="48" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="47" t="n"/>
+      <c r="B13" s="47" t="n"/>
+      <c r="C13" s="48" t="inlineStr">
         <is>
           <t>TOTAL PROYECTO</t>
         </is>
       </c>
-      <c r="D12" s="47" t="n"/>
-      <c r="E12" s="47" t="n"/>
-      <c r="F12" s="49">
-        <f>SUM(F4:F7)+F10</f>
-        <v/>
-      </c>
-      <c r="G12" s="21">
-        <f>SUM(G4:G7)+G10</f>
-        <v/>
-      </c>
-      <c r="H12" s="21">
-        <f>SUM(H4:H7)+H10</f>
-        <v/>
-      </c>
-      <c r="I12" s="22">
-        <f>SUM(I4:I7)+I10</f>
-        <v/>
-      </c>
-      <c r="J12" s="23">
-        <f>SUM(J4:J7)+J10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="D13" s="47" t="n"/>
+      <c r="E13" s="47" t="n"/>
+      <c r="F13" s="49">
+        <f>SUM(F4:F8)+F11</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>SUM(G4:G8)+G11</f>
+        <v/>
+      </c>
+      <c r="H13" s="21">
+        <f>SUM(H4:H8)+H11</f>
+        <v/>
+      </c>
+      <c r="I13" s="22">
+        <f>SUM(I4:I8)+I11</f>
+        <v/>
+      </c>
+      <c r="J13" s="23">
+        <f>SUM(J4:J8)+J11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Las columnas 'Horas' e 'Importe' se calculan solas a partir de la hoja Sesiones. No escribas en ellas.</t>
         </is>

</xml_diff>

<commit_message>
cifrado y hashing, arreglo vista
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO.xlsx
+++ b/SEGUIMIENTO.xlsx
@@ -942,7 +942,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una) a partir de las marcas de tiempo de los archivos y del volumen de los commits. Del 15 de agosto en adelante estan registradas en tiempo real. Total pendiente de facturar: 21,2 h = 424 EUR.</t>
+          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una). Del 15 de agosto en adelante registradas en tiempo real. Total pendiente de facturar: 24,2 h = 484 EUR.</t>
         </is>
       </c>
     </row>
@@ -1583,14 +1583,42 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="n"/>
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="33" t="n"/>
-      <c r="F14" s="34" t="n"/>
-      <c r="G14" s="34" t="n"/>
-      <c r="H14" s="34" t="n"/>
+      <c r="A14" s="32" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>BC-1</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>Evidencia al estandar bodycam, validado en la unidad: identidad del oficial en overlay + manifest (Officer.kt hardcodeado con TODO), un solo MP4 por incidente (IncidentAssembler, remux sin recodificar), rotulo del oficial quemado en los frames (VideoStamper, decode-GL-encode por hardware; el firmware no trae watermark), nombres placa_fecha_hora, numeracion secuencial INC_000001 con contador auto-reparable, .nomedia en el anillo</t>
+        </is>
+      </c>
+      <c r="F14" s="50" t="inlineStr">
+        <is>
+          <t>671cab7, 48892dd, b00332f, 4373116, a25c0c7</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="57" t="inlineStr">
+        <is>
+          <t>Marcas de tiempo 19:06-21:05</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -2059,7 +2087,7 @@
       </c>
       <c r="E4" s="37" t="inlineStr">
         <is>
-          <t>Integrado en develop (06008b2) y validado en la unidad</t>
+          <t>Al estandar bodycam (video unico con rotulo), validado en la unidad</t>
         </is>
       </c>
       <c r="F4" s="10" t="n">
@@ -2676,7 +2704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2738,12 +2766,12 @@
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
-          <t>f2e7e52</t>
+          <t>a25c0c7</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
         <is>
-          <t>armar al abrir la app - la pieza de 56d5478 que no llego al disco</t>
+          <t>numeracion secuencial INC_000001 con contador auto-reparable</t>
         </is>
       </c>
       <c r="E4" s="38" t="inlineStr">
@@ -2763,12 +2791,12 @@
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>99b42a6</t>
+          <t>4373116</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>LED por estado real: el azul de buffer ya no se pisa con verde</t>
+          <t>rotulo del oficial quemado en los frames + .nomedia en el anillo</t>
         </is>
       </c>
       <c r="E5" s="38" t="inlineStr">
@@ -2788,12 +2816,12 @@
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>2ecc7d5</t>
+          <t>b00332f</t>
         </is>
       </c>
       <c r="D6" s="28" t="inlineStr">
         <is>
-          <t>pre buffer integrado, led azul y armar al abrir la app (seguimiento)</t>
+          <t>un incidente = un unico MP4, ensamblado sin recodificar</t>
         </is>
       </c>
       <c r="E6" s="38" t="inlineStr">
@@ -2813,12 +2841,12 @@
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>56d5478</t>
+          <t>48892dd</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>buffer automatico al abrir, pre-roll de 20 s y LED azul en servicio</t>
+          <t>evidencia con nombre placa_fecha_hora al promoverse</t>
         </is>
       </c>
       <c r="E7" s="38" t="inlineStr">
@@ -2838,12 +2866,12 @@
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>06008b2</t>
+          <t>671cab7</t>
         </is>
       </c>
       <c r="D8" s="28" t="inlineStr">
         <is>
-          <t>merge main: grabacion continua con pre-roll sobre la UI nueva de develop</t>
+          <t>identidad del oficial en overlay y manifest</t>
         </is>
       </c>
       <c r="E8" s="38" t="inlineStr">
@@ -2863,12 +2891,12 @@
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>a599da9</t>
+          <t>16c498a</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>botones en pantalla quitados, prebuffer mejorado, ux y enviar a servidor</t>
+          <t>arreglos (usuario)</t>
         </is>
       </c>
       <c r="E9" s="38" t="inlineStr">
@@ -2888,12 +2916,12 @@
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>db04e55</t>
+          <t>f2e7e52</t>
         </is>
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>botones de subir a server</t>
+          <t>armar al abrir la app - la pieza de 56d5478 que no llego al disco</t>
         </is>
       </c>
       <c r="E10" s="38" t="inlineStr">
@@ -2904,7 +2932,7 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46249</v>
+        <v>46257</v>
       </c>
       <c r="B11" s="31" t="inlineStr">
         <is>
@@ -2913,12 +2941,12 @@
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
-          <t>420590e</t>
+          <t>99b42a6</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>no segmentacion, pantalla cerrada al grabar, cronometro</t>
+          <t>LED por estado real: el azul de buffer ya no se pisa con verde</t>
         </is>
       </c>
       <c r="E11" s="38" t="inlineStr">
@@ -2929,7 +2957,7 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46243</v>
+        <v>46257</v>
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
@@ -2938,12 +2966,12 @@
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>d4a4709</t>
+          <t>2ecc7d5</t>
         </is>
       </c>
       <c r="D12" s="28" t="inlineStr">
         <is>
-          <t>avance grabacion continua</t>
+          <t>pre buffer integrado, led azul y armar al abrir la app (seguimiento)</t>
         </is>
       </c>
       <c r="E12" s="38" t="inlineStr">
@@ -2953,133 +2981,133 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="n">
-        <v>46225</v>
-      </c>
-      <c r="B13" s="34" t="inlineStr">
-        <is>
-          <t>AeriaNexusPrototype</t>
-        </is>
-      </c>
-      <c r="C13" s="50" t="inlineStr">
-        <is>
-          <t>74cba54</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
-        <is>
-          <t>quitado screenrecorder bloqueo</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="A13" s="4" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>56d5478</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="inlineStr">
+        <is>
+          <t>buffer automatico al abrir, pre-roll de 20 s y LED azul en servicio</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46223</v>
+        <v>46257</v>
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>AeriaNexusPrototype</t>
+          <t>BodyCamServer</t>
         </is>
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>327f4a6</t>
+          <t>06008b2</t>
         </is>
       </c>
       <c r="D14" s="28" t="inlineStr">
         <is>
-          <t>ahora las versiones debug aumentan automaticamente</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>merge main: grabacion continua con pre-roll sobre la UI nueva de develop</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="n">
-        <v>46223</v>
-      </c>
-      <c r="B15" s="34" t="inlineStr">
-        <is>
-          <t>AeriaNexusPrototype</t>
-        </is>
-      </c>
-      <c r="C15" s="50" t="inlineStr">
-        <is>
-          <t>82adb88</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>guardado local de incidencias</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="A15" s="4" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>a599da9</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>botones en pantalla quitados, prebuffer mejorado, ux y enviar a servidor</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46218</v>
+        <v>46257</v>
       </c>
       <c r="B16" s="31" t="inlineStr">
         <is>
-          <t>AeriaNexusPrototype</t>
+          <t>BodyCamServer</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
         <is>
-          <t>21c325e</t>
+          <t>db04e55</t>
         </is>
       </c>
       <c r="D16" s="28" t="inlineStr">
         <is>
-          <t>screenshot bloqueado, tooltip SOS, topbar no clickable, icono de mapa en SOS</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>botones de subir a server</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="32" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="A17" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>BodyCamServer</t>
         </is>
       </c>
-      <c r="C17" s="50" t="inlineStr">
-        <is>
-          <t>98cea82</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
-        <is>
-          <t>gitignore</t>
-        </is>
-      </c>
-      <c r="E17" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>420590e</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>no segmentacion, pantalla cerrada al grabar, cronometro</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46215</v>
+        <v>46243</v>
       </c>
       <c r="B18" s="31" t="inlineStr">
         <is>
@@ -3088,23 +3116,23 @@
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
-          <t>116a4c7</t>
+          <t>d4a4709</t>
         </is>
       </c>
       <c r="D18" s="28" t="inlineStr">
         <is>
-          <t>arreglos de grabacion desde telefono</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>avance grabacion continua</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="32" t="n">
-        <v>46215</v>
+        <v>46225</v>
       </c>
       <c r="B19" s="34" t="inlineStr">
         <is>
@@ -3113,12 +3141,12 @@
       </c>
       <c r="C19" s="50" t="inlineStr">
         <is>
-          <t>46c1f9e</t>
+          <t>74cba54</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>camara video bodycam</t>
+          <t>quitado screenrecorder bloqueo</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -3129,21 +3157,21 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46215</v>
+        <v>46223</v>
       </c>
       <c r="B20" s="31" t="inlineStr">
         <is>
-          <t>BodyCamServer</t>
+          <t>AeriaNexusPrototype</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>b69cc42</t>
+          <t>327f4a6</t>
         </is>
       </c>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>bluetooth arreglado y funcionalidad de camara</t>
+          <t>ahora las versiones debug aumentan automaticamente</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -3154,7 +3182,7 @@
     </row>
     <row r="21">
       <c r="A21" s="32" t="n">
-        <v>46215</v>
+        <v>46223</v>
       </c>
       <c r="B21" s="34" t="inlineStr">
         <is>
@@ -3163,12 +3191,12 @@
       </c>
       <c r="C21" s="50" t="inlineStr">
         <is>
-          <t>a772f1c</t>
+          <t>82adb88</t>
         </is>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>foto controlador desde el movil SOS, tooltip</t>
+          <t>guardado local de incidencias</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -3179,7 +3207,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="B22" s="31" t="inlineStr">
         <is>
@@ -3188,12 +3216,12 @@
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>6bfbd55</t>
+          <t>21c325e</t>
         </is>
       </c>
       <c r="D22" s="28" t="inlineStr">
         <is>
-          <t>Initial commit</t>
+          <t>screenshot bloqueado, tooltip SOS, topbar no clickable, icono de mapa en SOS</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -3204,7 +3232,7 @@
     </row>
     <row r="23">
       <c r="A23" s="32" t="n">
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="B23" s="34" t="inlineStr">
         <is>
@@ -3213,12 +3241,12 @@
       </c>
       <c r="C23" s="50" t="inlineStr">
         <is>
-          <t>d8a50e8</t>
+          <t>98cea82</t>
         </is>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>arreglado bug de bluetooth</t>
+          <t>gitignore</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -3229,7 +3257,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46190</v>
+        <v>46215</v>
       </c>
       <c r="B24" s="31" t="inlineStr">
         <is>
@@ -3238,12 +3266,12 @@
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>560756c</t>
+          <t>116a4c7</t>
         </is>
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>arreglo luces e icono</t>
+          <t>arreglos de grabacion desde telefono</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -3254,21 +3282,21 @@
     </row>
     <row r="25">
       <c r="A25" s="32" t="n">
-        <v>46189</v>
+        <v>46215</v>
       </c>
       <c r="B25" s="34" t="inlineStr">
         <is>
-          <t>BodyCamServer</t>
+          <t>AeriaNexusPrototype</t>
         </is>
       </c>
       <c r="C25" s="50" t="inlineStr">
         <is>
-          <t>8210f65</t>
+          <t>46c1f9e</t>
         </is>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
-          <t>icono agregado</t>
+          <t>camara video bodycam</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -3279,7 +3307,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46177</v>
+        <v>46215</v>
       </c>
       <c r="B26" s="31" t="inlineStr">
         <is>
@@ -3288,12 +3316,12 @@
       </c>
       <c r="C26" s="29" t="inlineStr">
         <is>
-          <t>cf69bcd</t>
+          <t>b69cc42</t>
         </is>
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>avanzada y arreglada</t>
+          <t>bluetooth arreglado y funcionalidad de camara</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -3304,21 +3332,21 @@
     </row>
     <row r="27">
       <c r="A27" s="32" t="n">
-        <v>46175</v>
+        <v>46215</v>
       </c>
       <c r="B27" s="34" t="inlineStr">
         <is>
-          <t>BodyCamServer</t>
+          <t>AeriaNexusPrototype</t>
         </is>
       </c>
       <c r="C27" s="50" t="inlineStr">
         <is>
-          <t>16f3d49</t>
+          <t>a772f1c</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>arreglo blue y botones</t>
+          <t>foto controlador desde el movil SOS, tooltip</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
@@ -3329,21 +3357,21 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46139</v>
+        <v>46213</v>
       </c>
       <c r="B28" s="31" t="inlineStr">
         <is>
-          <t>BodyCamServer</t>
+          <t>AeriaNexusPrototype</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>eb63e85</t>
+          <t>6bfbd55</t>
         </is>
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>muy funcional, falta layout de pantalla de estado</t>
+          <t>Initial commit</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
@@ -3354,7 +3382,7 @@
     </row>
     <row r="29">
       <c r="A29" s="32" t="n">
-        <v>46137</v>
+        <v>46213</v>
       </c>
       <c r="B29" s="34" t="inlineStr">
         <is>
@@ -3363,12 +3391,12 @@
       </c>
       <c r="C29" s="50" t="inlineStr">
         <is>
-          <t>4797b0a</t>
+          <t>d8a50e8</t>
         </is>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>arreglo server</t>
+          <t>arreglado bug de bluetooth</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -3379,7 +3407,7 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46135</v>
+        <v>46190</v>
       </c>
       <c r="B30" s="31" t="inlineStr">
         <is>
@@ -3388,12 +3416,12 @@
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>c99cd77</t>
+          <t>560756c</t>
         </is>
       </c>
       <c r="D30" s="28" t="inlineStr">
         <is>
-          <t>new upload</t>
+          <t>arreglo luces e icono</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -3404,32 +3432,166 @@
     </row>
     <row r="31">
       <c r="A31" s="32" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B31" s="55" t="n"/>
+      <c r="C31" s="55" t="n"/>
+      <c r="D31" s="55" t="n"/>
+      <c r="E31" s="56" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>cf69bcd</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>avanzada y arreglada</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C33" s="50" t="inlineStr">
+        <is>
+          <t>16f3d49</t>
+        </is>
+      </c>
+      <c r="D33" s="33" t="inlineStr">
+        <is>
+          <t>arreglo blue y botones</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>eb63e85</t>
+        </is>
+      </c>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>muy funcional, falta layout de pantalla de estado</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B35" s="34" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="inlineStr">
+        <is>
+          <t>4797b0a</t>
+        </is>
+      </c>
+      <c r="D35" s="33" t="inlineStr">
+        <is>
+          <t>arreglo server</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
         <v>46135</v>
       </c>
-      <c r="B31" s="34" t="inlineStr">
+      <c r="B36" s="31" t="inlineStr">
         <is>
           <t>BodyCamServer</t>
         </is>
       </c>
-      <c r="C31" s="50" t="inlineStr">
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>c99cd77</t>
+        </is>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>new upload</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="inlineStr">
         <is>
           <t>60448a3</t>
         </is>
       </c>
-      <c r="D31" s="33" t="inlineStr">
+      <c r="D37" s="33" t="inlineStr">
         <is>
           <t>first commit</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="51" t="inlineStr">
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="51" t="inlineStr">
         <is>
           <t>Total: 20 commits · 13 días naturales con actividad (BodyCamServer 10 · AeriaNexus 5 · 2 días compartidos)</t>
         </is>

</xml_diff>

<commit_message>
cifrado de conexion con bodycam
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO.xlsx
+++ b/SEGUIMIENTO.xlsx
@@ -21,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -218,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -355,6 +356,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -799,11 +801,11 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>30 dias desde el pago</t>
+          <t>32 dias desde el pago</t>
         </is>
       </c>
     </row>
@@ -869,14 +871,14 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>BC-1, BC-2, BC-3, BC-4, ADM</t>
+          <t>BC-1, BC-2, BC-3, BC-4, BC-5, ADM</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>4900</v>
+        <v>6860</v>
       </c>
       <c r="F13" s="12">
         <f>SUMIFS(Sesiones!$D:$D,Sesiones!$B:$B,"BC",Sesiones!$A:$A,"&gt;="&amp;DATE(2026,7,24))</f>
@@ -895,14 +897,14 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AN-1</t>
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0</v>
+        <v>799</v>
       </c>
       <c r="F14" s="17">
         <f>SUMIFS(Sesiones!$D:$D,Sesiones!$B:$B,"AN",Sesiones!$A:$A,"&gt;="&amp;DATE(2026,7,24))</f>
@@ -920,7 +922,7 @@
         </is>
       </c>
       <c r="C15" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D15" s="20">
         <f>SUM(D13:D14)</f>
@@ -942,7 +944,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una). Del 15 de agosto en adelante registradas en tiempo real. Total pendiente de facturar: 24,2 h = 484 EUR.</t>
+          <t>Horas del 09 y 14 de agosto reconstruidas a posteriori (6,0 h cada una). Del 15 de agosto en adelante registradas en tiempo real. El 25 de agosto es el primer dia desde el pago con trabajo en las DOS aplicaciones. Total pendiente de facturar: 26,7 h = 534 EUR.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1066,7 @@
       </c>
       <c r="C28" s="26" t="inlineStr">
         <is>
-          <t>BC-2 es medición previa al cifrado, no una funcionalidad terminada. Convendría facturarlo como investigación, no como feature entregada.</t>
+          <t>BC-2 es medicion previa al cifrado, no una funcionalidad terminada; convendria facturarlo como investigacion. La funcionalidad si esta terminada en BC-5 (25-ago): la evidencia sale cifrada y hasheada de la unidad, validado en hardware. BLOQUEADO por decision del manager: custodia de la clave. Hasta que llegue la publica de Nexus la subida envia el MP4 en claro a proposito, porque el servidor no podria abrir un .fev cifrado solo para el Keystore de la unidad.</t>
         </is>
       </c>
       <c r="D28" s="55" t="n"/>
@@ -1083,7 +1085,7 @@
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Registrado a 2026-08-23</t>
+          <t>Registrado a 2026-08-25</t>
         </is>
       </c>
       <c r="C31">
@@ -1127,7 +1129,7 @@
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>A 30 h/semana las horas restantes se cubren en ~2,7 semanas: el umbral de 2000 EUR se cruza alrededor del jueves 10 de septiembre de 2026. La ventana 24-ago -&gt; 30-sep (5 semanas + 3 dias) da capacidad para 168 h = hasta 187 h acumuladas = 3740 EUR.</t>
+          <t>A 30 h/semana las 73,3 h restantes se cubren en ~2,4 semanas: el umbral de 2000 EUR se cruza alrededor del viernes 11 de septiembre de 2026. La ventana 25-ago -&gt; 30-sep (5 semanas + 1 dia) da capacidad para ~154 h = hasta ~181 h acumuladas = ~3614 EUR.</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1621,24 +1623,80 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="27" t="n"/>
-      <c r="E15" s="28" t="n"/>
-      <c r="F15" s="31" t="n"/>
-      <c r="G15" s="31" t="n"/>
-      <c r="H15" s="31" t="n"/>
+      <c r="A15" s="32" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>BC-5</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Cifrado y hash de la evidencia (IMPLEMENTACION): formato FEVD v1 documentado como contrato de las dos apps (docs/CRYPTO-FORMAT.md), EvidenceCrypto (AES-256-GCM en bloques de 1 MB con nonce y AAD derivados del indice, mas SHA-256 en la misma pasada), EvidenceKeys (DEK por fichero + envoltorios: Keystore del dispositivo funcional, RSA-OAEP del servidor listo y desactivado), hashes persistidos en el manifest, disparo al cerrar el incidente, descifrador Python de referencia. Validado en la unidad: 20,3 MB cifrados en 397 ms, descifrado en PC identico byte a byte. Version 1.2 (versionCode 3)</t>
+        </is>
+      </c>
+      <c r="F15" s="50" t="inlineStr">
+        <is>
+          <t>81f0995</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="57" t="inlineStr">
+        <is>
+          <t>Marcas de tiempo 12:30-15:00</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="n"/>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="33" t="n"/>
-      <c r="F16" s="34" t="n"/>
-      <c r="G16" s="34" t="n"/>
-      <c r="H16" s="34" t="n"/>
+      <c r="A16" s="32" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>AN-1</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Cifrado y hash de la evidencia (PORT AL TELEFONO): EvidenceCrypto y EvidenceKeys identicos byte a byte a los de la bodycam salvo el alias de Keystore, enganche al cerrar la captura, .fev a almacenamiento privado (fuera de la galeria), hashes simulados sustituidos por SHA-256 real. Compila; sin validar en telefono</t>
+        </is>
+      </c>
+      <c r="F16" s="50" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" s="57" t="inlineStr">
+        <is>
+          <t>Marcas de tiempo 12:43-12:58</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -1940,7 +1998,6 @@
       <c r="G46" s="34" t="n"/>
       <c r="H46" s="34" t="n"/>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="C48" s="35" t="inlineStr">
         <is>
@@ -1952,17 +2009,6 @@
         <v/>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -1992,7 +2038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2277,109 +2323,154 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="39" t="n"/>
-      <c r="B9" s="39" t="n"/>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>BC-5</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>BodyCamServer</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>Cifrado y hash de la evidencia (implementacion)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>En develop (81f0995), validado en la unidad. Version 1.2 en codigo; la unidad corre el binario 1.1 (mismo codigo, compilado antes del salto)</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>1060</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="12">
+        <f>SUMIF(Sesiones!$C:$C,A9,Sesiones!$D:$D)</f>
+        <v/>
+      </c>
+      <c r="J9" s="13">
+        <f>I9*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="39" t="n"/>
+      <c r="B10" s="39" t="n"/>
+      <c r="C10" s="40" t="inlineStr">
         <is>
           <t>Subtotal BodyCamServer</t>
         </is>
       </c>
-      <c r="D9" s="39" t="n"/>
-      <c r="E9" s="39" t="n"/>
-      <c r="F9" s="41">
-        <f>SUM(F4:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="42">
-        <f>SUM(G4:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="42">
-        <f>SUM(H4:H8)</f>
-        <v/>
-      </c>
-      <c r="I9" s="43">
-        <f>SUM(I4:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="44">
-        <f>SUM(J4:J8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="36" t="inlineStr">
-        <is>
-          <t>AN</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="inlineStr">
+      <c r="D10" s="39" t="n"/>
+      <c r="E10" s="39" t="n"/>
+      <c r="F10" s="41">
+        <f>SUM(F4:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="42">
+        <f>SUM(G4:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="42">
+        <f>SUM(H4:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="43">
+        <f>SUM(I4:I9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="44">
+        <f>SUM(J4:J9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
+          <t>AN-1</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>AeriaNexusPrototype</t>
         </is>
       </c>
-      <c r="C11" s="45" t="inlineStr">
-        <is>
-          <t>Sin bloques posteriores al pago</t>
-        </is>
-      </c>
-      <c r="D11" s="31" t="n"/>
-      <c r="E11" s="37" t="inlineStr">
-        <is>
-          <t>Al día</t>
-        </is>
-      </c>
-      <c r="F11" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="13">
-        <f>I10*Resumen!$C$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="47" t="n"/>
-      <c r="B13" s="47" t="n"/>
-      <c r="C13" s="48" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
+        <is>
+          <t>Cifrado y hash de la evidencia (port de FEVD v1)</t>
+        </is>
+      </c>
+      <c r="D12" s="58" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>Sin commitear. Compila; sin validar en telefono</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>799</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="I12" s="12">
+        <f>SUMIF(Sesiones!$C:$C,A12,Sesiones!$D:$D)</f>
+        <v/>
+      </c>
+      <c r="J12" s="13">
+        <f>I12*Resumen!$C$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="47" t="n"/>
+      <c r="B14" s="47" t="n"/>
+      <c r="C14" s="48" t="inlineStr">
         <is>
           <t>TOTAL PROYECTO</t>
         </is>
       </c>
-      <c r="D13" s="47" t="n"/>
-      <c r="E13" s="47" t="n"/>
-      <c r="F13" s="49">
-        <f>SUM(F4:F8)+F11</f>
-        <v/>
-      </c>
-      <c r="G13" s="21">
-        <f>SUM(G4:G8)+G11</f>
-        <v/>
-      </c>
-      <c r="H13" s="21">
-        <f>SUM(H4:H8)+H11</f>
-        <v/>
-      </c>
-      <c r="I13" s="22">
-        <f>SUM(I4:I8)+I11</f>
-        <v/>
-      </c>
-      <c r="J13" s="23">
-        <f>SUM(J4:J8)+J11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="D14" s="47" t="n"/>
+      <c r="E14" s="47" t="n"/>
+      <c r="F14" s="49">
+        <f>SUM(F4:F9)+F12</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>SUM(G4:G9)+G12</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>SUM(H4:H9)+H12</f>
+        <v/>
+      </c>
+      <c r="I14" s="22">
+        <f>SUM(I4:I9)+I12</f>
+        <v/>
+      </c>
+      <c r="J14" s="23">
+        <f>SUM(J4:J9)+J12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Las columnas 'Horas' e 'Importe' se calculan solas a partir de la hoja Sesiones. No escribas en ellas.</t>
         </is>
@@ -2387,8 +2478,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A15:J15"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A14:J14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3284,26 +3375,10 @@
       <c r="A25" s="32" t="n">
         <v>46215</v>
       </c>
-      <c r="B25" s="34" t="inlineStr">
-        <is>
-          <t>AeriaNexusPrototype</t>
-        </is>
-      </c>
-      <c r="C25" s="50" t="inlineStr">
-        <is>
-          <t>46c1f9e</t>
-        </is>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
-        <is>
-          <t>camara video bodycam</t>
-        </is>
-      </c>
-      <c r="E25" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B25" s="55" t="n"/>
+      <c r="C25" s="55" t="n"/>
+      <c r="D25" s="55" t="n"/>
+      <c r="E25" s="56" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -3589,7 +3664,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="51" t="inlineStr">
         <is>

</xml_diff>